<commit_message>
feat: sync current medication workbook skill
</commit_message>
<xml_diff>
--- a/assets/medication-reminder-template.xlsx
+++ b/assets/medication-reminder-template.xlsx
@@ -2,9 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rc3319cdaf0c34203"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R410bf13cb67443ea"/>
   </x:sheets>
 </x:workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -283,106 +287,81 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="8" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="34" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="12" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="8" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="8" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="20" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="36" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="24" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="22" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="68" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="12" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="18" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="20" hidden="0" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>用药提醒服务明细</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>序号</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>患者唯一标识</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>姓名</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>性别</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>年龄</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>疾病</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>既往过敏史</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="str">
-        <v>手术名称</v>
-      </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>联合用药</t>
-        </is>
-      </c>
-      <c r="J2" s="6" t="inlineStr">
-        <is>
-          <t>用药方案确认时间</t>
-        </is>
-      </c>
-      <c r="K2" s="6" t="inlineStr">
-        <is>
-          <t>用药方案</t>
-        </is>
-      </c>
-      <c r="L2" s="6" t="inlineStr">
-        <is>
-          <t>用药周期</t>
-        </is>
-      </c>
-      <c r="M2" s="6" t="inlineStr">
-        <is>
-          <t>方案链接</t>
-        </is>
-      </c>
-      <c r="N2" s="6" t="inlineStr">
-        <is>
-          <t>本月是否发生不良反应（AE）</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells>
-    <mergeCell ref="A1:N1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="8" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="68" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>用药提醒服务明细</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="42" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B2" s="6" t="str">
+        <x:v>患者唯一标识</x:v>
+      </x:c>
+      <x:c r="C2" s="6" t="str">
+        <x:v>姓名</x:v>
+      </x:c>
+      <x:c r="D2" s="6" t="str">
+        <x:v>性别</x:v>
+      </x:c>
+      <x:c r="E2" s="6" t="str">
+        <x:v>年龄</x:v>
+      </x:c>
+      <x:c r="F2" s="6" t="str">
+        <x:v>疾病</x:v>
+      </x:c>
+      <x:c r="G2" s="6" t="str">
+        <x:v>既往过敏史</x:v>
+      </x:c>
+      <x:c r="H2" s="6" t="str">
+        <x:v>手术名称</x:v>
+      </x:c>
+      <x:c r="I2" s="6" t="str">
+        <x:v>耗材名称</x:v>
+      </x:c>
+      <x:c r="J2" s="6" t="str">
+        <x:v>联合用药</x:v>
+      </x:c>
+      <x:c r="K2" s="6" t="str">
+        <x:v>用药方案确认时间</x:v>
+      </x:c>
+      <x:c r="L2" s="6" t="str">
+        <x:v>用药方案</x:v>
+      </x:c>
+      <x:c r="M2" s="6" t="str">
+        <x:v>用药周期</x:v>
+      </x:c>
+      <x:c r="N2" s="6" t="str">
+        <x:v>方案链接</x:v>
+      </x:c>
+      <x:c r="O2" t="str">
+        <x:v>本月是否发生不良反应（AE）</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:O1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: preserve monthly source metadata
</commit_message>
<xml_diff>
--- a/assets/medication-reminder-template.xlsx
+++ b/assets/medication-reminder-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R410bf13cb67443ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R4599fd5ad6ea47ed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -334,33 +334,42 @@
         <x:v>既往过敏史</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str">
+        <x:v>用户类型</x:v>
+      </x:c>
+      <x:c r="I2" s="6" t="str">
+        <x:v>来源任务ID</x:v>
+      </x:c>
+      <x:c r="J2" s="6" t="str">
+        <x:v>来源月份</x:v>
+      </x:c>
+      <x:c r="K2" s="6" t="str">
         <x:v>手术名称</x:v>
       </x:c>
-      <x:c r="I2" s="6" t="str">
+      <x:c r="L2" s="6" t="str">
         <x:v>耗材名称</x:v>
       </x:c>
-      <x:c r="J2" s="6" t="str">
+      <x:c r="M2" s="6" t="str">
         <x:v>联合用药</x:v>
       </x:c>
-      <x:c r="K2" s="6" t="str">
+      <x:c r="N2" s="6" t="str">
         <x:v>用药方案确认时间</x:v>
       </x:c>
-      <x:c r="L2" s="6" t="str">
+      <x:c r="O2" t="str">
         <x:v>用药方案</x:v>
       </x:c>
-      <x:c r="M2" s="6" t="str">
+      <x:c r="P2" t="str">
         <x:v>用药周期</x:v>
       </x:c>
-      <x:c r="N2" s="6" t="str">
+      <x:c r="Q2" t="str">
         <x:v>方案链接</x:v>
       </x:c>
-      <x:c r="O2" t="str">
+      <x:c r="R2" t="str">
         <x:v>本月是否发生不良反应（AE）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:O1"/>
+    <x:mergeCell ref="A1:R1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>